<commit_message>
add Defect doc and update TestCase doc
</commit_message>
<xml_diff>
--- a/20130199_TestDesign.xlsx
+++ b/20130199_TestDesign.xlsx
@@ -1371,7 +1371,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="25.5" spans="1:6">
+    <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
@@ -1572,7 +1572,7 @@
       </c>
       <c r="F17" s="5"/>
     </row>
-    <row r="18" ht="38.25" spans="1:6">
+    <row r="18" ht="25.5" spans="1:6">
       <c r="A18" s="7"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="F59" s="5"/>
     </row>
-    <row r="60" ht="38.25" spans="1:6">
+    <row r="60" ht="25.5" spans="1:6">
       <c r="A60" s="7"/>
       <c r="B60" s="7"/>
       <c r="C60" s="7"/>

</xml_diff>